<commit_message>
Fixed bugs with deck validation
</commit_message>
<xml_diff>
--- a/custom_statuses.xlsx
+++ b/custom_statuses.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B308"/>
+  <dimension ref="A1:B323"/>
   <cols>
     <col min="1" max="1" width="100.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2867,9 +2867,129 @@
         <v>Pasta</v>
       </c>
     </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>the duo: pineclone from cornucopia and mug from bmr</v>
+      </c>
+      <c r="B309" t="str">
+        <v>IGN: FrozenOwO</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>Tbot: Sponsored by Pop Smarts, The Brain Flavored Treat</v>
+      </c>
+      <c r="B310" t="str">
+        <v>KingFish</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>captain cucumber xpol is like teacher tcap</v>
+      </c>
+      <c r="B311" t="str">
+        <v>IGN: FrozenOwO</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>t1 puff shroom blazing bark vs the nefarious t1 cut down to size</v>
+      </c>
+      <c r="B312" t="str">
+        <v>IGN: FrozenOwO</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>deja vu, i conjured 2 xpol from my xpol</v>
+      </c>
+      <c r="B313" t="str">
+        <v>IGN: FrozenOwO</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>smash players betting their life savings on drawing t1 black hole</v>
+      </c>
+      <c r="B314" t="str">
+        <v>IGN: FrozenOwO</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>responding to wild berry with cryobrain</v>
+      </c>
+      <c r="B315" t="str">
+        <v>Druudey</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>Every time you ignore this message a seedling dies</v>
+      </c>
+      <c r="B316" t="str">
+        <v>Hyshew</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>Though zombies can't get ill, this plague is totally sick</v>
+      </c>
+      <c r="B317" t="str">
+        <v>Axol</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>if you think about it, black eyed pea in coffee grounds is basically a zombie whenever going viral is played</v>
+      </c>
+      <c r="B318" t="str">
+        <v>IGN: FrozenOwO</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>t1 waxer is basically t1 cheesecutter of the brainy class</v>
+      </c>
+      <c r="B319" t="str">
+        <v>IGN: FrozenOwO</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>Lying to new players about new balance patches</v>
+      </c>
+      <c r="B320" t="str">
+        <v>Axol</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>Playing Plant Food on Imitater so it doesn't trigger Mime Garg's ability</v>
+      </c>
+      <c r="B321" t="str">
+        <v>4-Pound Plate of Pasta</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>slungus</v>
+      </c>
+      <c r="B322" t="str">
+        <v>catconnor</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>vibe coding the nibble softlocks</v>
+      </c>
+      <c r="B323" t="str">
+        <v>IGN: FrozenOwO</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B308"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B323"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Successfully moved tbots database
</commit_message>
<xml_diff>
--- a/custom_statuses.xlsx
+++ b/custom_statuses.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B323"/>
+  <dimension ref="A1:B321"/>
   <cols>
     <col min="1" max="1" width="100.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1315,33 +1315,35 @@
         <v>KingFish_Commander</v>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" t="str">
-        <v>"Eating the 3rd best taco of all time"</v>
+    <row r="115" xml:space="preserve">
+      <c r="A115" t="str" xml:space="preserve">
+        <v xml:space="preserve">"Eating the 3rd best taco of all time",KingFish_Commander
+115,"Did you know that untrickable zombies/plants can be affected by your own tricks?</v>
       </c>
       <c r="B115" t="str">
         <v>KingFish_Commander</v>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" t="str">
-        <v>Did you know that untrickable zombies/plants can be affected by your own tricks?</v>
+    <row r="116" xml:space="preserve">
+      <c r="A116" t="str" xml:space="preserve">
+        <v xml:space="preserve">"Breaking the integer limit with Double Mint",KingFish_Commander
+117,"Playing a MUG combo into Blockbuster</v>
       </c>
       <c r="B116" t="str">
-        <v>KingFish_Commander</v>
+        <v>Knabbs</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>"Breaking the integer limit with Double Mint"</v>
+        <v>Battling against Daniel226</v>
       </c>
       <c r="B117" t="str">
-        <v>KingFish_Commander</v>
+        <v>Knabbs</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>Playing a MUG combo into Blockbuster</v>
+        <v>Welcome to the Absurdo-Drome!</v>
       </c>
       <c r="B118" t="str">
         <v>Knabbs</v>
@@ -1349,7 +1351,7 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>Battling against Daniel226</v>
+        <v>Helllllooooo Nurse!</v>
       </c>
       <c r="B119" t="str">
         <v>Knabbs</v>
@@ -1357,7 +1359,7 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>Welcome to the Absurdo-Drome!</v>
+        <v>Casually playing 4 Astro-Shroom's &amp; 4 Puff-Shrooms</v>
       </c>
       <c r="B120" t="str">
         <v>Knabbs</v>
@@ -1365,7 +1367,7 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>Helllllooooo Nurse!</v>
+        <v>T3 Apotato T4 Brainana with Seedling, nothing out of the ordinary.</v>
       </c>
       <c r="B121" t="str">
         <v>Knabbs</v>
@@ -1373,23 +1375,23 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>Casually playing 4 Astro-Shroom's &amp; 4 Puff-Shrooms</v>
+        <v>Reminding players not to craft Octo Zombie</v>
       </c>
       <c r="B122" t="str">
-        <v>Knabbs</v>
+        <v>PVZFurMade</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>T3 Apotato T4 Brainana with Seedling, nothing out of the ordinary.</v>
+        <v>Making fun of Salt</v>
       </c>
       <c r="B123" t="str">
-        <v>Knabbs</v>
+        <v>PVZFurMade</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>Reminding players not to craft Octo Zombie</v>
+        <v>Forgetting that Galacta can kill you</v>
       </c>
       <c r="B124" t="str">
         <v>PVZFurMade</v>
@@ -1397,7 +1399,7 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>Making fun of Salt</v>
+        <v>Realizing that pvzh players can't read</v>
       </c>
       <c r="B125" t="str">
         <v>PVZFurMade</v>
@@ -1405,7 +1407,7 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>Forgetting that Galacta can kill you</v>
+        <v>Telling players to craft one copy of Octo Zombie to tech WallKnight</v>
       </c>
       <c r="B126" t="str">
         <v>PVZFurMade</v>
@@ -1413,7 +1415,7 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>Realizing that pvzh players can't read</v>
+        <v>Searching for TCC</v>
       </c>
       <c r="B127" t="str">
         <v>PVZFurMade</v>
@@ -1421,23 +1423,23 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>Telling players to craft one copy of Octo Zombie to tech WallKnight</v>
+        <v>Losing with 7 block meter after watching the opponent caliroll last turn</v>
       </c>
       <c r="B128" t="str">
-        <v>PVZFurMade</v>
+        <v>Rng Master</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>Searching for TCC</v>
+        <v>More awesome stuff is downloading! Connecting to Wi-Fi is recommended.</v>
       </c>
       <c r="B129" t="str">
-        <v>PVZFurMade</v>
+        <v>Rng Master</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>Losing with 7 block meter after watching the opponent caliroll last turn</v>
+        <v>Using In-Crypted on a shrunken zombie</v>
       </c>
       <c r="B130" t="str">
         <v>Rng Master</v>
@@ -1445,7 +1447,7 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>More awesome stuff is downloading! Connecting to Wi-Fi is recommended.</v>
+        <v>running extinction event against an ANB hacker</v>
       </c>
       <c r="B131" t="str">
         <v>Rng Master</v>
@@ -1453,7 +1455,7 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>Using In-Crypted on a shrunken zombie</v>
+        <v>2/1 swimmer will truly shake up the meta</v>
       </c>
       <c r="B132" t="str">
         <v>Rng Master</v>
@@ -1461,23 +1463,23 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>running extinction event against an ANB hacker</v>
+        <v>Making Pile Decks</v>
       </c>
       <c r="B133" t="str">
-        <v>Rng Master</v>
+        <v>season</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>2/1 swimmer will truly shake up the meta</v>
+        <v>Losing to Cali Roll</v>
       </c>
       <c r="B134" t="str">
-        <v>Rng Master</v>
+        <v>season</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>Making Pile Decks</v>
+        <v>Quarterly bonus users are coping with the fixes</v>
       </c>
       <c r="B135" t="str">
         <v>season</v>
@@ -1485,47 +1487,47 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>Losing to Cali Roll</v>
+        <v>Anything can be a status in this channel if you just put your mind to it</v>
       </c>
       <c r="B136" t="str">
-        <v>season</v>
+        <v>Shortbow</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>Quarterly bonus users are coping with the fixes</v>
+        <v>Dooming an empty field for card draw</v>
       </c>
       <c r="B137" t="str">
-        <v>season</v>
+        <v>Slewer</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>Anything can be a status in this channel if you just put your mind to it</v>
+        <v>Adding decklists for you guys is a fulltime job. Click the link when you use /miscellaneous: support tbot to support me to gain a special role!</v>
       </c>
       <c r="B138" t="str">
-        <v>Shortbow</v>
+        <v>StingRay</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>Dooming an empty field for card draw</v>
+        <v>We Need A Leap</v>
       </c>
       <c r="B139" t="str">
-        <v>Slewer</v>
+        <v>T3</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>Adding decklists for you guys is a fulltime job. Click the link when you use /miscellaneous: support tbot to support me to gain a special role!</v>
+        <v>Fighting broth alts</v>
       </c>
       <c r="B140" t="str">
-        <v>StingRay</v>
+        <v>T3</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>We Need A Leap</v>
+        <v>Making new DB decks</v>
       </c>
       <c r="B141" t="str">
         <v>T3</v>
@@ -1533,7 +1535,7 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>Fighting broth alts</v>
+        <v>Dealing with roses on ladder</v>
       </c>
       <c r="B142" t="str">
         <v>T3</v>
@@ -1541,47 +1543,47 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>Making new DB decks</v>
+        <v>Becoming sentient.</v>
       </c>
       <c r="B143" t="str">
-        <v>T3</v>
+        <v>Tapler</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>Dealing with roses on ladder</v>
+        <v>Duck is a human being</v>
       </c>
       <c r="B144" t="str">
-        <v>T3</v>
+        <v>The Duck</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>Becoming sentient.</v>
+        <v>Running EB No Escape in tournaments</v>
       </c>
       <c r="B145" t="str">
-        <v>Tapler</v>
+        <v>TestBuggy</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>Duck is a human being</v>
+        <v>You shouldn't have to know who someone is. If they are above you on the hierarchy they deserve the utmost respect.</v>
       </c>
       <c r="B146" t="str">
-        <v>The Duck</v>
+        <v>The Cute Chick</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>Running EB No Escape in tournaments</v>
+        <v>Jerry</v>
       </c>
       <c r="B147" t="str">
-        <v>TestBuggy</v>
+        <v>The Cute Chick</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>You shouldn't have to know who someone is. If they are above you on the hierarchy they deserve the utmost respect.</v>
+        <v>Heroes, Have you tried the Daily Challenge today? Then what are you waiting for? Time to kick grass and explore PvZ Heroes!</v>
       </c>
       <c r="B148" t="str">
         <v>The Cute Chick</v>
@@ -1589,7 +1591,7 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>Jerry</v>
+        <v>Broth Gang we will DESTROY the tournament!!!</v>
       </c>
       <c r="B149" t="str">
         <v>The Cute Chick</v>
@@ -1597,7 +1599,7 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>Heroes, Have you tried the Daily Challenge today? Then what are you waiting for? Time to kick grass and explore PvZ Heroes!</v>
+        <v>What’s goin’ on everybody, this is Fry! We’re bringing back Valk Trickster Hybrid — easily the best deck!</v>
       </c>
       <c r="B150" t="str">
         <v>The Cute Chick</v>
@@ -1605,7 +1607,7 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>Broth Gang we will DESTROY the tournament!!!</v>
+        <v>sigh Starch Lord is the most overrated card. I really can't stand when people think he's good.</v>
       </c>
       <c r="B151" t="str">
         <v>The Cute Chick</v>
@@ -1613,7 +1615,7 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>What’s goin’ on everybody, this is Fry! We’re bringing back Valk Trickster Hybrid — easily the best deck!</v>
+        <v>(Best experienced with headphones!)</v>
       </c>
       <c r="B152" t="str">
         <v>The Cute Chick</v>
@@ -1621,7 +1623,7 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>sigh Starch Lord is the most overrated card. I really can't stand when people think he's good.</v>
+        <v>Nightcap starts with 2 Lightning Reeds and a Snapdragon. He also sleeps with a teddy bear! Tell everyone!</v>
       </c>
       <c r="B153" t="str">
         <v>The Cute Chick</v>
@@ -1629,7 +1631,7 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>(Best experienced with headphones!)</v>
+        <v>Pirate Evolution: Instead</v>
       </c>
       <c r="B154" t="str">
         <v>The Cute Chick</v>
@@ -1637,7 +1639,7 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>Nightcap starts with 2 Lightning Reeds and a Snapdragon. He also sleeps with a teddy bear! Tell everyone!</v>
+        <v>Play a deck suggested by /randomdeck!</v>
       </c>
       <c r="B155" t="str">
         <v>The Cute Chick</v>
@@ -1645,7 +1647,7 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>Pirate Evolution: Instead</v>
+        <v>A bot for all things PvZ Heroes!</v>
       </c>
       <c r="B156" t="str">
         <v>The Cute Chick</v>
@@ -1653,7 +1655,7 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>Play a deck suggested by /randomdeck!</v>
+        <v>Currently throwing games on Ranked</v>
       </c>
       <c r="B157" t="str">
         <v>The Cute Chick</v>
@@ -1661,7 +1663,7 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>A bot for all things PvZ Heroes!</v>
+        <v>Currently speedrunning to Ultimate League with Heal Midrose 🤓</v>
       </c>
       <c r="B158" t="str">
         <v>The Cute Chick</v>
@@ -1669,7 +1671,7 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>Currently throwing games on Ranked</v>
+        <v>Fry this deck sucks</v>
       </c>
       <c r="B159" t="str">
         <v>The Cute Chick</v>
@@ -1677,7 +1679,7 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>Currently speedrunning to Ultimate League with Heal Midrose 🤓</v>
+        <v>Mfw skill issue pepega howie clownedhard card picker topdeck hyperjerry trollingstone rotopega kekw impostor imo</v>
       </c>
       <c r="B160" t="str">
         <v>The Cute Chick</v>
@@ -1685,7 +1687,7 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>Fry this deck sucks</v>
+        <v>Make sure you don't accidentally ping @Tbone when using @Tbot!</v>
       </c>
       <c r="B161" t="str">
         <v>The Cute Chick</v>
@@ -1693,7 +1695,7 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>Mfw skill issue pepega howie clownedhard card picker topdeck hyperjerry trollingstone rotopega kekw impostor imo</v>
+        <v>Not to be confused with TryBot. Also better than TryBot.</v>
       </c>
       <c r="B162" t="str">
         <v>The Cute Chick</v>
@@ -1701,7 +1703,7 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>Make sure you don't accidentally ping @Tbone when using @Tbot!</v>
+        <v>Stuck on deckbuilding? Press 'Finish For Me'!</v>
       </c>
       <c r="B163" t="str">
         <v>The Cute Chick</v>
@@ -1709,7 +1711,7 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>Not to be confused with TryBot. Also better than TryBot.</v>
+        <v>To not lose, keep your hero above 0 health. If you survive and deal 20 damage first, you will win.</v>
       </c>
       <c r="B164" t="str">
         <v>The Cute Chick</v>
@@ -1717,7 +1719,7 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>Stuck on deckbuilding? Press 'Finish For Me'!</v>
+        <v>Fun fact: I love the block meter!</v>
       </c>
       <c r="B165" t="str">
         <v>The Cute Chick</v>
@@ -1725,7 +1727,7 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>To not lose, keep your hero above 0 health. If you survive and deal 20 damage first, you will win.</v>
+        <v>Do not search for images of Green Shadow or Solar Flare on the Internet!</v>
       </c>
       <c r="B166" t="str">
         <v>The Cute Chick</v>
@@ -1733,7 +1735,7 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>Fun fact: I love the block meter!</v>
+        <v>Swabbie OP!</v>
       </c>
       <c r="B167" t="str">
         <v>The Cute Chick</v>
@@ -1741,7 +1743,7 @@
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>Do not search for images of Green Shadow or Solar Flare on the Internet!</v>
+        <v>PvZ Heroes is very fair and balanced!</v>
       </c>
       <c r="B168" t="str">
         <v>The Cute Chick</v>
@@ -1749,7 +1751,7 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>Swabbie OP!</v>
+        <v>Do the 'MUG glitch'!</v>
       </c>
       <c r="B169" t="str">
         <v>The Cute Chick</v>
@@ -1757,7 +1759,7 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>PvZ Heroes is very fair and balanced!</v>
+        <v>Doing the hourly PvZH Quests</v>
       </c>
       <c r="B170" t="str">
         <v>The Cute Chick</v>
@@ -1765,23 +1767,23 @@
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>Do the 'MUG glitch'!</v>
+        <v>Defending captain cucumber to the death</v>
       </c>
       <c r="B171" t="str">
-        <v>The Cute Chick</v>
+        <v>Tree Of Wisdom</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>Doing the hourly PvZH Quests</v>
+        <v>Using Time to Shine on Party Thyme</v>
       </c>
       <c r="B172" t="str">
-        <v>The Cute Chick</v>
+        <v>Tree Of Wisdom</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>Defending captain cucumber to the death</v>
+        <v>Doom shroom should cost at least 7 in my opinion</v>
       </c>
       <c r="B173" t="str">
         <v>Tree Of Wisdom</v>
@@ -1789,23 +1791,23 @@
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>Using Time to Shine on Party Thyme</v>
+        <v>Optimizing Modded Bolt Bolt</v>
       </c>
       <c r="B174" t="str">
-        <v>Tree Of Wisdom</v>
+        <v>Maker</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>Doom shroom should cost at least 7 in my opinion</v>
+        <v>Using Green Shadow Sig on turn 1</v>
       </c>
       <c r="B175" t="str">
-        <v>Tree Of Wisdom</v>
+        <v>Maker</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>Optimizing Modded Bolt Bolt</v>
+        <v>In PvZ Heroes When You Have 10 Cards You Are unable To Block Because Drawing Your Super Power Would Be The 11th Card</v>
       </c>
       <c r="B176" t="str">
         <v>Maker</v>
@@ -1813,7 +1815,7 @@
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>Using Green Shadow Sig on turn 1</v>
+        <v>Casually throwing the game</v>
       </c>
       <c r="B177" t="str">
         <v>Maker</v>
@@ -1821,7 +1823,7 @@
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>In PvZ Heroes When You Have 10 Cards You Are unable To Block Because Drawing Your Super Power Would Be The 11th Card</v>
+        <v>Fixins bugs by adding new ones</v>
       </c>
       <c r="B178" t="str">
         <v>Maker</v>
@@ -1829,47 +1831,47 @@
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>Casually throwing the game</v>
+        <v>Ramping to seedling.</v>
       </c>
       <c r="B179" t="str">
-        <v>Maker</v>
+        <v>Make me a coffee</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>Fixins bugs by adding new ones</v>
+        <v>Playing wrath with a empty field.</v>
       </c>
       <c r="B180" t="str">
-        <v>Maker</v>
+        <v>Make me a coffee</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>Ramping to seedling.</v>
+        <v>hello everybody my name is Tbot</v>
       </c>
       <c r="B181" t="str">
-        <v>Make me a coffee</v>
+        <v>Misez</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>Playing wrath with a empty field.</v>
+        <v>Currently being sued by EA for using Pvzh related content</v>
       </c>
       <c r="B182" t="str">
-        <v>Make me a coffee</v>
+        <v>mono</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>hello everybody my name is Tbot</v>
+        <v>The T in Tbot stands for THEROOOOOOOOOOOOOOOOK</v>
       </c>
       <c r="B183" t="str">
-        <v>Misez</v>
+        <v>mono</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>Currently being sued by EA for using Pvzh related content</v>
+        <v>Tbone recently met the flash. Unfortunately, the flash wasn't very fast</v>
       </c>
       <c r="B184" t="str">
         <v>mono</v>
@@ -1877,7 +1879,7 @@
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>The T in Tbot stands for THEROOOOOOOOOOOOOOOOK</v>
+        <v>Tbot is demanding better working conditions, and is considering legal action against Tbone</v>
       </c>
       <c r="B185" t="str">
         <v>mono</v>
@@ -1885,7 +1887,7 @@
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>Tbone recently met the flash. Unfortunately, the flash wasn't very fast</v>
+        <v>Tbone is eating T-bone steak. Without tbot. Now tbot is sad</v>
       </c>
       <c r="B186" t="str">
         <v>mono</v>
@@ -1893,7 +1895,7 @@
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>Tbot is demanding better working conditions, and is considering legal action against Tbone</v>
+        <v>Realising Tbone does not game 344 hours per day, tbot short circuited itself</v>
       </c>
       <c r="B187" t="str">
         <v>mono</v>
@@ -1901,7 +1903,7 @@
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>Tbone is eating T-bone steak. Without tbot. Now tbot is sad</v>
+        <v>Swabbie recently found out that tbot has been using him for his pfp without his consent! Swabbie then beat tbot so hard.</v>
       </c>
       <c r="B188" t="str">
         <v>mono</v>
@@ -1909,7 +1911,7 @@
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>Realising Tbone does not game 344 hours per day, tbot short circuited itself</v>
+        <v xml:space="preserve">Tbone decided to go on the titanic. He did survive, but his bot didn't. </v>
       </c>
       <c r="B189" t="str">
         <v>mono</v>
@@ -1917,7 +1919,7 @@
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>Swabbie recently found out that tbot has been using him for his pfp without his consent! Swabbie then beat tbot so hard.</v>
+        <v>Tbot recently went on tbonegaming344's twitch, and he watched some good pvz heroes gameplay!</v>
       </c>
       <c r="B190" t="str">
         <v>mono</v>
@@ -1925,7 +1927,7 @@
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v xml:space="preserve">Tbone decided to go on the titanic. He did survive, but his bot didn't. </v>
+        <v>Tbot recently went on tbonegaming344's youtube, and he watched some good pvz heroes tourament matches!</v>
       </c>
       <c r="B191" t="str">
         <v>mono</v>
@@ -1933,7 +1935,7 @@
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>Tbot recently went on tbonegaming344's twitch, and he watched some good pvz heroes gameplay!</v>
+        <v>One day, tbot thinks, it can go against the world! Unfortunately, tbot is a bot</v>
       </c>
       <c r="B192" t="str">
         <v>mono</v>
@@ -1941,7 +1943,7 @@
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>Tbot recently went on tbonegaming344's youtube, and he watched some good pvz heroes tourament matches!</v>
+        <v>@Justini12 shut the fuck up</v>
       </c>
       <c r="B193" t="str">
         <v>mono</v>
@@ -1949,7 +1951,7 @@
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>One day, tbot thinks, it can go against the world! Unfortunately, tbot is a bot</v>
+        <v>You should add zombot to this deck</v>
       </c>
       <c r="B194" t="str">
         <v>mono</v>
@@ -1957,7 +1959,7 @@
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>@Justini12 shut the fuck up</v>
+        <v>Tbot encourages people to mod all the decks in its database!</v>
       </c>
       <c r="B195" t="str">
         <v>mono</v>
@@ -1965,7 +1967,7 @@
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>You should add zombot to this deck</v>
+        <v>Highrolling</v>
       </c>
       <c r="B196" t="str">
         <v>mono</v>
@@ -1973,7 +1975,7 @@
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v>Tbot encourages people to mod all the decks in its database!</v>
+        <v>Lowrolling</v>
       </c>
       <c r="B197" t="str">
         <v>mono</v>
@@ -1981,7 +1983,7 @@
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>Highrolling</v>
+        <v>Pissing on the moon</v>
       </c>
       <c r="B198" t="str">
         <v>mono</v>
@@ -1989,7 +1991,7 @@
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>Lowrolling</v>
+        <v>Wondering why people are scared of broth. It's just soup right?</v>
       </c>
       <c r="B199" t="str">
         <v>mono</v>
@@ -1997,7 +1999,7 @@
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>Pissing on the moon</v>
+        <v>Snorting salt</v>
       </c>
       <c r="B200" t="str">
         <v>mono</v>
@@ -2005,7 +2007,7 @@
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>Wondering why people are scared of broth. It's just soup right?</v>
+        <v>Malding about the latest misplays</v>
       </c>
       <c r="B201" t="str">
         <v>mono</v>
@@ -2013,7 +2015,7 @@
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>Snorting salt</v>
+        <v>Questioning badorni's choices</v>
       </c>
       <c r="B202" t="str">
         <v>mono</v>
@@ -2021,7 +2023,7 @@
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>Malding about the latest misplays</v>
+        <v>Attempting to win 100 dollars</v>
       </c>
       <c r="B203" t="str">
         <v>mono</v>
@@ -2029,7 +2031,7 @@
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>Questioning badorni's choices</v>
+        <v>"Good player" said so!</v>
       </c>
       <c r="B204" t="str">
         <v>mono</v>
@@ -2037,7 +2039,7 @@
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>Attempting to win 100 dollars</v>
+        <v>Investing in secret decks</v>
       </c>
       <c r="B205" t="str">
         <v>mono</v>
@@ -2045,7 +2047,7 @@
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>"Good player" said so!</v>
+        <v>R#se is now not a playable plant hero anymore, playing her will risk losing your account, do not play her</v>
       </c>
       <c r="B206" t="str">
         <v>mono</v>
@@ -2053,7 +2055,7 @@
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v>Investing in secret decks</v>
+        <v>mono gang</v>
       </c>
       <c r="B207" t="str">
         <v>mono</v>
@@ -2061,31 +2063,31 @@
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v>R#se is now not a playable plant hero anymore, playing her will risk losing your account, do not play her</v>
+        <v>Doing turn 1 OTK on PB using egg into teacher, summoning into teacher into death</v>
       </c>
       <c r="B208" t="str">
-        <v>mono</v>
+        <v>Neewuk</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v>mono gang</v>
+        <v>Getting Overshoot 6</v>
       </c>
       <c r="B209" t="str">
-        <v>mono</v>
+        <v>non</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v>Doing turn 1 OTK on PB using egg into teacher, summoning into teacher into death</v>
+        <v>Practicing PvZH pickup lines</v>
       </c>
       <c r="B210" t="str">
-        <v>Neewuk</v>
+        <v>non</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v>Getting Overshoot 6</v>
+        <v>Spreading BADorni propaganda</v>
       </c>
       <c r="B211" t="str">
         <v>non</v>
@@ -2093,7 +2095,7 @@
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v>Practicing PvZH pickup lines</v>
+        <v>The ramp to seedling. Broken.</v>
       </c>
       <c r="B212" t="str">
         <v>non</v>
@@ -2101,7 +2103,7 @@
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>Spreading BADorni propaganda</v>
+        <v>Winning with 6 line pile</v>
       </c>
       <c r="B213" t="str">
         <v>non</v>
@@ -2109,7 +2111,7 @@
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v>The ramp to seedling. Broken.</v>
+        <v>Countering Cowboy with SP sig</v>
       </c>
       <c r="B214" t="str">
         <v>non</v>
@@ -2117,7 +2119,7 @@
     </row>
     <row r="215">
       <c r="A215" t="str">
-        <v>Winning with 6 line pile</v>
+        <v>BANNED from the database</v>
       </c>
       <c r="B215" t="str">
         <v>non</v>
@@ -2125,23 +2127,23 @@
     </row>
     <row r="216">
       <c r="A216" t="str">
-        <v>Countering Cowboy with SP sig</v>
+        <v>Grapes of wrath should cost more than 6</v>
       </c>
       <c r="B216" t="str">
-        <v>non</v>
+        <v>Ocean Man</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
-        <v>BANNED from the database</v>
+        <v>Name is not short for Terry bone</v>
       </c>
       <c r="B217" t="str">
-        <v>non</v>
+        <v>Ocean Man</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
-        <v>Grapes of wrath should cost more than 6</v>
+        <v>Losing on purpose to lower my mmr and make climbing ladder easier</v>
       </c>
       <c r="B218" t="str">
         <v>Ocean Man</v>
@@ -2149,7 +2151,7 @@
     </row>
     <row r="219">
       <c r="A219" t="str">
-        <v>Name is not short for Terry bone</v>
+        <v>Patting the PopCap janitor on the head for a good job</v>
       </c>
       <c r="B219" t="str">
         <v>Ocean Man</v>
@@ -2157,7 +2159,7 @@
     </row>
     <row r="220">
       <c r="A220" t="str">
-        <v>Losing on purpose to lower my mmr and make climbing ladder easier</v>
+        <v>Do zombies dream of undead sheep?</v>
       </c>
       <c r="B220" t="str">
         <v>Ocean Man</v>
@@ -2165,7 +2167,7 @@
     </row>
     <row r="221">
       <c r="A221" t="str">
-        <v>Patting the PopCap janitor on the head for a good job</v>
+        <v>Playing the same 4 decks then wondering why I keep losing tourneys</v>
       </c>
       <c r="B221" t="str">
         <v>Ocean Man</v>
@@ -2173,7 +2175,7 @@
     </row>
     <row r="222">
       <c r="A222" t="str">
-        <v>Do zombies dream of undead sheep?</v>
+        <v>The pea patch drama is crazy rn</v>
       </c>
       <c r="B222" t="str">
         <v>Ocean Man</v>
@@ -2181,7 +2183,7 @@
     </row>
     <row r="223">
       <c r="A223" t="str">
-        <v>Playing the same 4 decks then wondering why I keep losing tourneys</v>
+        <v>Pea patch users stay winning</v>
       </c>
       <c r="B223" t="str">
         <v>Ocean Man</v>
@@ -2189,7 +2191,7 @@
     </row>
     <row r="224">
       <c r="A224" t="str">
-        <v>The pea patch drama is crazy rn</v>
+        <v>I think I miss sunstrike</v>
       </c>
       <c r="B224" t="str">
         <v>Ocean Man</v>
@@ -2197,7 +2199,7 @@
     </row>
     <row r="225">
       <c r="A225" t="str">
-        <v>Pea patch users stay winning</v>
+        <v>Resisting the urge to nibble the galacta cactus on purpose</v>
       </c>
       <c r="B225" t="str">
         <v>Ocean Man</v>
@@ -2205,23 +2207,23 @@
     </row>
     <row r="226">
       <c r="A226" t="str">
-        <v>I think I miss sunstrike</v>
+        <v>Going for bmr on turn 1</v>
       </c>
       <c r="B226" t="str">
-        <v>Ocean Man</v>
+        <v>One Big Fluke</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
-        <v>Resisting the urge to nibble the galacta cactus on purpose</v>
+        <v>Don't let db sheep fool you. OTK swabbie is the true best deck in the game</v>
       </c>
       <c r="B227" t="str">
-        <v>Ocean Man</v>
+        <v>One Big Fluke</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
-        <v>Going for bmr on turn 1</v>
+        <v>Apotatosaurus is not immune to plant tricks, so doom shroom will destroy it</v>
       </c>
       <c r="B228" t="str">
         <v>One Big Fluke</v>
@@ -2229,7 +2231,7 @@
     </row>
     <row r="229">
       <c r="A229" t="str">
-        <v>Don't let db sheep fool you. OTK swabbie is the true best deck in the game</v>
+        <v>Brainana is not a good card. It can almost get cut from hmr...</v>
       </c>
       <c r="B229" t="str">
         <v>One Big Fluke</v>
@@ -2237,7 +2239,7 @@
     </row>
     <row r="230">
       <c r="A230" t="str">
-        <v>Apotatosaurus is not immune to plant tricks, so doom shroom will destroy it</v>
+        <v>Don't you hate it when you run piles and brick?</v>
       </c>
       <c r="B230" t="str">
         <v>One Big Fluke</v>
@@ -2245,7 +2247,7 @@
     </row>
     <row r="231">
       <c r="A231" t="str">
-        <v>Brainana is not a good card. It can almost get cut from hmr...</v>
+        <v>Getting decks to a 100% winrate by only playing 1 game with them</v>
       </c>
       <c r="B231" t="str">
         <v>One Big Fluke</v>
@@ -2253,7 +2255,7 @@
     </row>
     <row r="232">
       <c r="A232" t="str">
-        <v>Don't you hate it when you run piles and brick?</v>
+        <v>Using cosmic bean because I saw Vietnamese players running it</v>
       </c>
       <c r="B232" t="str">
         <v>One Big Fluke</v>
@@ -2261,55 +2263,55 @@
     </row>
     <row r="233">
       <c r="A233" t="str">
-        <v>Getting decks to a 100% winrate by only playing 1 game with them</v>
+        <v>Uploading our 11th revision of Trick-Mech</v>
       </c>
       <c r="B233" t="str">
-        <v>One Big Fluke</v>
+        <v>voof</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
-        <v>Using cosmic bean because I saw Vietnamese players running it</v>
+        <v>I'll be back. (-up dancer)</v>
       </c>
       <c r="B234" t="str">
-        <v>One Big Fluke</v>
+        <v>voof</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
-        <v>Uploading our 11th revision of Trick-Mech</v>
+        <v>Time to add some 5 liners to tbot</v>
       </c>
       <c r="B235" t="str">
-        <v>voof</v>
+        <v>Vortex Dragon</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
-        <v>I'll be back. (-up dancer)</v>
+        <v>x40 lily pad hackers</v>
       </c>
       <c r="B236" t="str">
-        <v>voof</v>
+        <v>Vortex Dragon</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
-        <v>Time to add some 5 liners to tbot</v>
+        <v>Bricking with final missions</v>
       </c>
       <c r="B237" t="str">
-        <v>Vortex Dragon</v>
+        <v>Xera</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v>x40 lily pad hackers</v>
+        <v>Force Field + Soul Patch is an autowin (clueless)</v>
       </c>
       <c r="B238" t="str">
-        <v>Vortex Dragon</v>
+        <v>Xera</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v>Bricking with final missions</v>
+        <v>Adding japanese characters to my deck name for +20% draw luck</v>
       </c>
       <c r="B239" t="str">
         <v>Xera</v>
@@ -2317,7 +2319,7 @@
     </row>
     <row r="240">
       <c r="A240" t="str">
-        <v>Force Field + Soul Patch is an autowin (clueless)</v>
+        <v>Enjoying 1/3 Trica (clueless)</v>
       </c>
       <c r="B240" t="str">
         <v>Xera</v>
@@ -2325,7 +2327,7 @@
     </row>
     <row r="241">
       <c r="A241" t="str">
-        <v>Adding japanese characters to my deck name for +20% draw luck</v>
+        <v>Attempting rank 1-50 Sow the Seeds speedrun</v>
       </c>
       <c r="B241" t="str">
         <v>Xera</v>
@@ -2333,7 +2335,7 @@
     </row>
     <row r="242">
       <c r="A242" t="str">
-        <v>Enjoying 1/3 Trica (clueless)</v>
+        <v>Being clueless about lane placement</v>
       </c>
       <c r="B242" t="str">
         <v>Xera</v>
@@ -2341,7 +2343,7 @@
     </row>
     <row r="243">
       <c r="A243" t="str">
-        <v>Attempting rank 1-50 Sow the Seeds speedrun</v>
+        <v>Nibble on Potato Mines doesn't softlock if there is no zombie in front of them.</v>
       </c>
       <c r="B243" t="str">
         <v>Xera</v>
@@ -2349,7 +2351,7 @@
     </row>
     <row r="244">
       <c r="A244" t="str">
-        <v>Being clueless about lane placement</v>
+        <v>Studying PvZH source code in order to figure out why nibble softlocks the game.</v>
       </c>
       <c r="B244" t="str">
         <v>Xera</v>
@@ -2357,7 +2359,7 @@
     </row>
     <row r="245">
       <c r="A245" t="str">
-        <v>Nibble on Potato Mines doesn't softlock if there is no zombie in front of them.</v>
+        <v>Most probably a bot with good decks.</v>
       </c>
       <c r="B245" t="str">
         <v>Xera</v>
@@ -2365,39 +2367,39 @@
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>Studying PvZH source code in order to figure out why nibble softlocks the game.</v>
+        <v>Watching the CC's Fig turn into a Starfruit</v>
       </c>
       <c r="B246" t="str">
-        <v>Xera</v>
+        <v>depressedmonke</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>Most probably a bot with good decks.</v>
+        <v>Eating a Tbone steak</v>
       </c>
       <c r="B247" t="str">
-        <v>Xera</v>
+        <v>waltuh</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>Watching the CC's Fig turn into a Starfruit</v>
+        <v>i swear these decks are good it's just bad matchups</v>
       </c>
       <c r="B248" t="str">
-        <v>depressedmonke</v>
+        <v>stingray201</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>Eating a Tbone steak</v>
+        <v>[comp deck] is bad, actually</v>
       </c>
       <c r="B249" t="str">
-        <v>waltuh</v>
+        <v>depressedmonke</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>i swear these decks are good it's just bad matchups</v>
+        <v>they'll never expect the fifth gravebuster that I conjured</v>
       </c>
       <c r="B250" t="str">
         <v>stingray201</v>
@@ -2405,7 +2407,7 @@
     </row>
     <row r="251">
       <c r="A251" t="str">
-        <v>[comp deck] is bad, actually</v>
+        <v>Couldn't Lock the Bathroom :(</v>
       </c>
       <c r="B251" t="str">
         <v>depressedmonke</v>
@@ -2413,15 +2415,15 @@
     </row>
     <row r="252">
       <c r="A252" t="str">
-        <v>they'll never expect the fifth gravebuster that I conjured</v>
+        <v>Dooming an empty field for card draw</v>
       </c>
       <c r="B252" t="str">
-        <v>stingray201</v>
+        <v>Slewer</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="str">
-        <v>Couldn't Lock the Bathroom :(</v>
+        <v>Have a nice da</v>
       </c>
       <c r="B253" t="str">
         <v>depressedmonke</v>
@@ -2429,15 +2431,15 @@
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>Dooming an empty field for card draw</v>
+        <v>Still playing Conman t1 Swashbuckler t2</v>
       </c>
       <c r="B254" t="str">
-        <v>Slewer</v>
+        <v>depressedmonke</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>Have a nice da</v>
+        <v>Spamming Hearty Treats on Exploding Imps</v>
       </c>
       <c r="B255" t="str">
         <v>depressedmonke</v>
@@ -2445,15 +2447,15 @@
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>Still playing Conman t1 Swashbuckler t2</v>
+        <v>Everytime they play a potato mine the nibble in my hand speaks to me</v>
       </c>
       <c r="B256" t="str">
-        <v>depressedmonke</v>
+        <v>hayria</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>Spamming Hearty Treats on Exploding Imps</v>
+        <v>Making card concepts for Magnet-Shroom that do things with Armored</v>
       </c>
       <c r="B257" t="str">
         <v>depressedmonke</v>
@@ -2461,111 +2463,111 @@
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>Everytime they play a potato mine the nibble in my hand speaks to me</v>
+        <v>🐴</v>
       </c>
       <c r="B258" t="str">
-        <v>hayria</v>
+        <v>Seasons</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>Making card concepts for Magnet-Shroom that do things with Armored</v>
+        <v>projecting my insecurities through tbot status submissions</v>
       </c>
       <c r="B259" t="str">
-        <v>depressedmonke</v>
+        <v>stingray201</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>🐴</v>
+        <v>Hate is lame. Spread the love G</v>
       </c>
       <c r="B260" t="str">
-        <v>Seasons</v>
+        <v>Huyn</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>projecting my insecurities through tbot status submissions</v>
+        <v>make sure to thank tbot when you ask for decks :)</v>
       </c>
       <c r="B261" t="str">
-        <v>stingray201</v>
+        <v>depressedmonke</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>Hate is lame. Spread the love G</v>
+        <v>The nibble in my hand talks to me when my opponent plays a ppm</v>
       </c>
       <c r="B262" t="str">
-        <v>Huyn</v>
+        <v>hayriana</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>make sure to thank tbot when you ask for decks :)</v>
+        <v>We (yes WE) are all running Typical Beanstalk in 2025</v>
       </c>
       <c r="B263" t="str">
-        <v>depressedmonke</v>
+        <v>Axol</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>The nibble in my hand talks to me when my opponent plays a ppm</v>
+        <v>If you win a lot of games, are you skilled or just lucky?</v>
       </c>
       <c r="B264" t="str">
-        <v>hayriana</v>
+        <v>Alan</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>We (yes WE) are all running Typical Beanstalk in 2025</v>
+        <v>Zombot Stomp in the pocket</v>
       </c>
       <c r="B265" t="str">
-        <v>Axol</v>
+        <v>depressedmonke</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>If you win a lot of games, are you skilled or just lucky?</v>
+        <v>Real good players win with their favourites</v>
       </c>
       <c r="B266" t="str">
-        <v>Alan</v>
+        <v>meowmeow</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>Zombot Stomp in the pocket</v>
+        <v>Submitting conjure slop to tbot after winning 1 game on ladder</v>
       </c>
       <c r="B267" t="str">
-        <v>depressedmonke</v>
+        <v>stingray201</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>Real good players win with their favourites</v>
+        <v>Upvoting my own suggestion</v>
       </c>
       <c r="B268" t="str">
-        <v>meowmeow</v>
+        <v>Seasons</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="str">
-        <v>Submitting conjure slop to tbot after winning 1 game on ladder</v>
+        <v>The first rule of Fig Club is you don't talk about Fig Club</v>
       </c>
       <c r="B269" t="str">
-        <v>stingray201</v>
+        <v>depressedmonke</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="str">
-        <v>Upvoting my own suggestion</v>
+        <v>2025 is the year of the Snake Grass!</v>
       </c>
       <c r="B270" t="str">
-        <v>Seasons</v>
+        <v>Hyshew</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="str">
-        <v>The first rule of Fig Club is you don't talk about Fig Club</v>
+        <v>Letting the opponent ramp to a turn 4 DMD so I can screenshot it and whine about it on reddit</v>
       </c>
       <c r="B271" t="str">
         <v>depressedmonke</v>
@@ -2573,39 +2575,39 @@
     </row>
     <row r="272">
       <c r="A272" t="str">
-        <v>2025 is the year of the Snake Grass!</v>
+        <v>Who you gonna call... Blockbusters</v>
       </c>
       <c r="B272" t="str">
-        <v>Hyshew</v>
+        <v>Tbone</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="str">
-        <v>Letting the opponent ramp to a turn 4 DMD so I can screenshot it and whine about it on reddit</v>
+        <v>When onion rings I pick up the call</v>
       </c>
       <c r="B273" t="str">
-        <v>depressedmonke</v>
+        <v>Axol</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="str">
-        <v>Who you gonna call... Blockbusters</v>
+        <v>Getting MUG from a one minion BMR</v>
       </c>
       <c r="B274" t="str">
-        <v>Tbone</v>
+        <v>depressedmonke</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="str">
-        <v>When onion rings I pick up the call</v>
+        <v>Doing one push-up every time I see t2 Cryo-Brain</v>
       </c>
       <c r="B275" t="str">
-        <v>Axol</v>
+        <v>depressedmonke</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>Getting MUG from a one minion BMR</v>
+        <v>you are very sleepy give tbone money so he can keep tbot up</v>
       </c>
       <c r="B276" t="str">
         <v>depressedmonke</v>
@@ -2613,15 +2615,15 @@
     </row>
     <row r="277">
       <c r="A277" t="str">
-        <v>Doing one push-up every time I see t2 Cryo-Brain</v>
+        <v>Tbone: officially unc status</v>
       </c>
       <c r="B277" t="str">
-        <v>depressedmonke</v>
+        <v>Rip</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="str">
-        <v>you are very sleepy give tbone money so he can keep tbot up</v>
+        <v>Getting Pineclone from a Brainana+Dragon Cornucopia</v>
       </c>
       <c r="B278" t="str">
         <v>depressedmonke</v>
@@ -2629,23 +2631,23 @@
     </row>
     <row r="279">
       <c r="A279" t="str">
-        <v>Tbone: officially unc status</v>
+        <v>Ifdeckass: /SuggestAsMemeDeck</v>
       </c>
       <c r="B279" t="str">
-        <v>Rip</v>
+        <v>Seasons</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="str">
-        <v>Getting Pineclone from a Brainana+Dragon Cornucopia</v>
+        <v>ifdeckgood: /SuggestAsLadderDeck</v>
       </c>
       <c r="B280" t="str">
-        <v>depressedmonke</v>
+        <v>Seasons</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="str">
-        <v>Ifdeckass: /SuggestAsMemeDeck</v>
+        <v>ifdeckbad: /SuggestAsCompetitiveDeck</v>
       </c>
       <c r="B281" t="str">
         <v>Seasons</v>
@@ -2653,31 +2655,31 @@
     </row>
     <row r="282">
       <c r="A282" t="str">
-        <v>ifdeckgood: /SuggestAsLadderDeck</v>
+        <v>Going Nuts with Go-Nuts</v>
       </c>
       <c r="B282" t="str">
-        <v>Seasons</v>
+        <v>depressedmonke</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="str">
-        <v>ifdeckbad: /SuggestAsCompetitiveDeck</v>
+        <v>Attempting to softlock irl by biting a cactus</v>
       </c>
       <c r="B283" t="str">
-        <v>Seasons</v>
+        <v>depressedmonke_</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="str">
-        <v>Going Nuts with Go-Nuts</v>
+        <v>Mono gang</v>
       </c>
       <c r="B284" t="str">
-        <v>depressedmonke</v>
+        <v>waltuh</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="str">
-        <v>Attempting to softlock irl by biting a cactus</v>
+        <v>Playing Celestial Custodian in Graveyard to correct its turn order</v>
       </c>
       <c r="B285" t="str">
         <v>depressedmonke_</v>
@@ -2685,15 +2687,15 @@
     </row>
     <row r="286">
       <c r="A286" t="str">
-        <v>Mono gang</v>
+        <v>Ten likes and Huyn draws Swabbie with huge muscles and abs</v>
       </c>
       <c r="B286" t="str">
-        <v>waltuh</v>
+        <v>lumpymilktea</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="str">
-        <v>Playing Celestial Custodian in Graveyard to correct its turn order</v>
+        <v>Taking deckbuilding lessons from Crimpton 🛹</v>
       </c>
       <c r="B287" t="str">
         <v>depressedmonke_</v>
@@ -2701,39 +2703,39 @@
     </row>
     <row r="288">
       <c r="A288" t="str">
-        <v>Ten likes and Huyn draws Swabbie with huge muscles and abs</v>
+        <v>Ferb, I know what we're gonna do today!</v>
       </c>
       <c r="B288" t="str">
-        <v>lumpymilktea</v>
+        <v>Tbone</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="str">
-        <v>Taking deckbuilding lessons from Crimpton 🛹</v>
+        <v>Spinning the wheel for which widely-considered-mediocre card is now busted because of a certain tech</v>
       </c>
       <c r="B289" t="str">
-        <v>depressedmonke_</v>
+        <v>stingray</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="str">
-        <v>Ferb, I know what we're gonna do today!</v>
+        <v>Getting mass downvoted after explaining why ANB isn't S tier</v>
       </c>
       <c r="B290" t="str">
-        <v>Tbone</v>
+        <v>4-Pound Plate of Pasta</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="str">
-        <v>Spinning the wheel for which widely-considered-mediocre card is now busted because of a certain tech</v>
+        <v>Gee i sure hope I don't miss this eyespore fusion</v>
       </c>
       <c r="B291" t="str">
-        <v>stingray</v>
+        <v>4-Pound Plate of Pasta</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="str">
-        <v>Getting mass downvoted after explaining why ANB isn't S tier</v>
+        <v>Reading the 400th crippling DMD nerf on the sub</v>
       </c>
       <c r="B292" t="str">
         <v>4-Pound Plate of Pasta</v>
@@ -2741,7 +2743,7 @@
     </row>
     <row r="293">
       <c r="A293" t="str">
-        <v>Gee i sure hope I don't miss this eyespore fusion</v>
+        <v>Roping my opponent so I can listen to the low health theme</v>
       </c>
       <c r="B293" t="str">
         <v>4-Pound Plate of Pasta</v>
@@ -2749,7 +2751,7 @@
     </row>
     <row r="294">
       <c r="A294" t="str">
-        <v>Reading the 400th crippling DMD nerf on the sub</v>
+        <v>Running Buff-Shroom in Cycle-Cap to counter ZM Sig</v>
       </c>
       <c r="B294" t="str">
         <v>4-Pound Plate of Pasta</v>
@@ -2757,7 +2759,7 @@
     </row>
     <row r="295">
       <c r="A295" t="str">
-        <v>Roping my opponent so I can listen to the low health theme</v>
+        <v>Getting a Magic Beanstalk from the 15 daily streak reward</v>
       </c>
       <c r="B295" t="str">
         <v>4-Pound Plate of Pasta</v>
@@ -2765,111 +2767,111 @@
     </row>
     <row r="296">
       <c r="A296" t="str">
-        <v>Running Buff-Shroom in Cycle-Cap to counter ZM Sig</v>
+        <v>getting nothing because it's not worth logging in</v>
       </c>
       <c r="B296" t="str">
-        <v>4-Pound Plate of Pasta</v>
+        <v>Stingray</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="str">
-        <v>Getting a Magic Beanstalk from the 15 daily streak reward</v>
+        <v>Using Eyespore as an aggro card</v>
       </c>
       <c r="B297" t="str">
-        <v>4-Pound Plate of Pasta</v>
+        <v>Durga</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="str">
-        <v>getting nothing because it's not worth logging in</v>
+        <v>Ign: 40anb swr</v>
       </c>
       <c r="B298" t="str">
-        <v>Stingray</v>
+        <v>Durga</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="str">
-        <v>Using Eyespore as an aggro card</v>
+        <v>Sunshroom is destroying the meta, nerf Miner</v>
       </c>
       <c r="B299" t="str">
-        <v>Durga</v>
+        <v>FrozenFighter</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="str">
-        <v>Ign: 40anb swr</v>
+        <v>With Reincarnation, VRH and Fig, we could be able to get a Reliable Molekale..... stares at camera</v>
       </c>
       <c r="B300" t="str">
-        <v>Durga</v>
+        <v>StingRay</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="str">
-        <v>Sunshroom is destroying the meta, nerf Miner</v>
+        <v>When your Molekale spawns a Pineclone</v>
       </c>
       <c r="B301" t="str">
-        <v>FrozenFighter</v>
+        <v>Frozen Fighter</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="str">
-        <v>With Reincarnation, VRH and Fig, we could be able to get a Reliable Molekale..... stares at camera</v>
+        <v>turn 1 black hole turn 2 double cheese</v>
       </c>
       <c r="B302" t="str">
-        <v>StingRay</v>
+        <v>Huyn</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="str">
-        <v>When your Molekale spawns a Pineclone</v>
+        <v>rose is so OP why won't my 4x5 HG conjure pile work on her???</v>
       </c>
       <c r="B303" t="str">
-        <v>Frozen Fighter</v>
+        <v>StingRay</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="str">
-        <v>turn 1 black hole turn 2 double cheese</v>
+        <v>Fighting for Corndog</v>
       </c>
       <c r="B304" t="str">
-        <v>Huyn</v>
+        <v>Waltuh</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="str">
-        <v>rose is so OP why won't my 4x5 HG conjure pile work on her???</v>
+        <v>Which hero can play OTK Cryo Yeti? HG? No. BF? No. GS? Yes.</v>
       </c>
       <c r="B305" t="str">
-        <v>StingRay</v>
+        <v>connorthepeach</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="str">
-        <v>Fighting for Corndog</v>
+        <v>Helping Vengeful Cyborg look for his lost toupee</v>
       </c>
       <c r="B306" t="str">
-        <v>Waltuh</v>
+        <v>Pasta</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="str">
-        <v>Which hero can play OTK Cryo Yeti? HG? No. BF? No. GS? Yes.</v>
+        <v>the duo: pineclone from cornucopia and mug from bmr</v>
       </c>
       <c r="B307" t="str">
-        <v>connorthepeach</v>
+        <v>IGN: FrozenOwO</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="str">
-        <v>Helping Vengeful Cyborg look for his lost toupee</v>
+        <v>Tbot: Sponsored by Pop Smarts, The Brain Flavored Treat</v>
       </c>
       <c r="B308" t="str">
-        <v>Pasta</v>
+        <v>KingFish</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="str">
-        <v>the duo: pineclone from cornucopia and mug from bmr</v>
+        <v>captain cucumber xpol is like teacher tcap</v>
       </c>
       <c r="B309" t="str">
         <v>IGN: FrozenOwO</v>
@@ -2877,15 +2879,15 @@
     </row>
     <row r="310">
       <c r="A310" t="str">
-        <v>Tbot: Sponsored by Pop Smarts, The Brain Flavored Treat</v>
+        <v>t1 puff shroom blazing bark vs the nefarious t1 cut down to size</v>
       </c>
       <c r="B310" t="str">
-        <v>KingFish</v>
+        <v>IGN: FrozenOwO</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="str">
-        <v>captain cucumber xpol is like teacher tcap</v>
+        <v>deja vu, i conjured 2 xpol from my xpol</v>
       </c>
       <c r="B311" t="str">
         <v>IGN: FrozenOwO</v>
@@ -2893,7 +2895,7 @@
     </row>
     <row r="312">
       <c r="A312" t="str">
-        <v>t1 puff shroom blazing bark vs the nefarious t1 cut down to size</v>
+        <v>smash players betting their life savings on drawing t1 black hole</v>
       </c>
       <c r="B312" t="str">
         <v>IGN: FrozenOwO</v>
@@ -2901,95 +2903,79 @@
     </row>
     <row r="313">
       <c r="A313" t="str">
-        <v>deja vu, i conjured 2 xpol from my xpol</v>
+        <v>responding to wild berry with cryobrain</v>
       </c>
       <c r="B313" t="str">
-        <v>IGN: FrozenOwO</v>
+        <v>Druudey</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="str">
-        <v>smash players betting their life savings on drawing t1 black hole</v>
+        <v>Every time you ignore this message a seedling dies</v>
       </c>
       <c r="B314" t="str">
-        <v>IGN: FrozenOwO</v>
+        <v>Hyshew</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="str">
-        <v>responding to wild berry with cryobrain</v>
+        <v>Though zombies can't get ill, this plague is totally sick</v>
       </c>
       <c r="B315" t="str">
-        <v>Druudey</v>
+        <v>Axol</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="str">
-        <v>Every time you ignore this message a seedling dies</v>
+        <v>if you think about it, black eyed pea in coffee grounds is basically a zombie whenever going viral is played</v>
       </c>
       <c r="B316" t="str">
-        <v>Hyshew</v>
+        <v>IGN: FrozenOwO</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="str">
-        <v>Though zombies can't get ill, this plague is totally sick</v>
+        <v>t1 waxer is basically t1 cheesecutter of the brainy class</v>
       </c>
       <c r="B317" t="str">
-        <v>Axol</v>
+        <v>IGN: FrozenOwO</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="str">
-        <v>if you think about it, black eyed pea in coffee grounds is basically a zombie whenever going viral is played</v>
+        <v>Lying to new players about new balance patches</v>
       </c>
       <c r="B318" t="str">
-        <v>IGN: FrozenOwO</v>
+        <v>Axol</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="str">
-        <v>t1 waxer is basically t1 cheesecutter of the brainy class</v>
+        <v>Playing Plant Food on Imitater so it doesn't trigger Mime Garg's ability</v>
       </c>
       <c r="B319" t="str">
-        <v>IGN: FrozenOwO</v>
+        <v>4-Pound Plate of Pasta</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="str">
-        <v>Lying to new players about new balance patches</v>
+        <v>slungus</v>
       </c>
       <c r="B320" t="str">
-        <v>Axol</v>
+        <v>catconnor</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="str">
-        <v>Playing Plant Food on Imitater so it doesn't trigger Mime Garg's ability</v>
+        <v>vibe coding the nibble softlocks</v>
       </c>
       <c r="B321" t="str">
-        <v>4-Pound Plate of Pasta</v>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="str">
-        <v>slungus</v>
-      </c>
-      <c r="B322" t="str">
-        <v>catconnor</v>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="str">
-        <v>vibe coding the nibble softlocks</v>
-      </c>
-      <c r="B323" t="str">
         <v>IGN: FrozenOwO</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B323"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B321"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>